<commit_message>
chore: verwijder School-specifieke importbestanden + neutraliseer voorbeelden
- Kluisgegevens.xlsx (170KB, 3385 kluisjes ISK School): eenmalig import-
  bestand, hoort niet in repo. Wordt straks ook uit git-history geschrubd
  via filter-repo.
- convert_isk_xlsx.py: eenmalig migratiescript voor ISK-data, niet
  relevant voor andere scholen.
- backend/voorbeeld-import.xlsx + frontend/public/voorbeeld-import.xlsx:
  "SCHOOL"-locatie-strings vervangen door "Hoofdgebouw". Dummy-
  namen (Jan/Emma/Sophie) behouden.

@
</commit_message>
<xml_diff>
--- a/backend/voorbeeld-import.xlsx
+++ b/backend/voorbeeld-import.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kluisgegevens" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Kluisjes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,23 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF8200"/>
-        <bgColor rgb="00FF8200"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,90 +415,74 @@
   </sheetPr>
   <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Cluster</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Kluis</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Naam</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Stamnummer</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Klas</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Uitleenperiode</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Borgbedrag</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Huurbedrag</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Locatie</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Sleutel</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Slot</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Studie</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Kluistype</t>
         </is>
@@ -565,7 +536,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>HET ERASMUS vestiging PrO</t>
+          <t>Hoofdgebouw - PrO</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -573,7 +544,6 @@
           <t>2040D</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>PRO 3</t>
@@ -633,7 +603,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>HET ERASMUS vestiging PrO</t>
+          <t>Hoofdgebouw - PrO</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -641,7 +611,6 @@
           <t>2656D</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>PRO 2</t>
@@ -664,9 +633,6 @@
           <t>P003</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>van - tot en met -</t>
@@ -689,7 +655,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>HET ERASMUS vestiging PrO</t>
+          <t>Hoofdgebouw - PrO</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -697,8 +663,6 @@
           <t>2723D</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>Leerlingkluisje</t>
@@ -753,7 +717,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>HET ERASMUS  -  MAVO/HAVO/VWO</t>
+          <t>Hoofdgebouw - MAVO/HAVO/VWO</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -761,7 +725,6 @@
           <t>X100</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>MAVO 4</t>
@@ -784,9 +747,6 @@
           <t>X101</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>van - tot en met -</t>
@@ -809,7 +769,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>HET ERASMUS  -  MAVO/HAVO/VWO</t>
+          <t>Hoofdgebouw - MAVO/HAVO/VWO</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -817,8 +777,6 @@
           <t>X101</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>Leerlingkluisje</t>

</xml_diff>